<commit_message>
Add 7-day and prior-day ROAS columns to product sheet
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-07-24.xlsx
+++ b/data/reports/report-2026-07-24.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -948,6 +948,13 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>・MER(7日)=Shopify売上(7日)÷Meta広告費(7日)。ROAS=Meta計上コンバージョン価値÷広告費（手計算値・Meta表示列は不使用）。前日ROASは単日値のためブレが大きく参考値</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -959,7 +966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -970,13 +977,15 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1022,35 +1031,45 @@
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
+          <t>前日ROAS</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
           <t>3日利益</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>30日利益</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
-        <is>
-          <t>MER</t>
-        </is>
-      </c>
       <c r="L1" s="3" t="inlineStr">
         <is>
+          <t>MER(7日)</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>ROAS(7日)</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
           <t>分岐</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>余裕</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>判定</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>予算</t>
         </is>
@@ -1083,27 +1102,33 @@
       <c r="H2" s="6" t="n">
         <v>0.435</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="I2" s="8" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="J2" s="5" t="n">
         <v>455982</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="K2" s="5" t="n">
         <v>2613247</v>
       </c>
-      <c r="K2" s="8" t="n">
+      <c r="L2" s="8" t="n">
         <v>4.36</v>
       </c>
-      <c r="L2" s="8" t="n">
+      <c r="M2" s="8" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="N2" s="8" t="n">
         <v>1.53</v>
       </c>
-      <c r="M2" s="8" t="n">
+      <c r="O2" s="8" t="n">
         <v>2.82</v>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>🎉記録更新（本日7/25判定）</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>85k維持</t>
         </is>
@@ -1136,27 +1161,33 @@
       <c r="H3" s="11" t="n">
         <v>0.357</v>
       </c>
-      <c r="I3" s="10" t="n">
+      <c r="I3" s="12" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="J3" s="10" t="n">
         <v>311271</v>
       </c>
-      <c r="J3" s="10" t="n">
+      <c r="K3" s="10" t="n">
         <v>2036918</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>3.24</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="N3" s="12" t="n">
         <v>1.35</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="O3" s="12" t="n">
         <v>1.88</v>
       </c>
-      <c r="N3" s="9" t="inlineStr">
+      <c r="P3" s="9" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="O3" s="9" t="inlineStr">
+      <c r="Q3" s="9" t="inlineStr">
         <is>
           <t>35k+25k維持</t>
         </is>
@@ -1189,27 +1220,33 @@
       <c r="H4" s="6" t="n">
         <v>0.356</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="I4" s="8" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="J4" s="5" t="n">
         <v>218426</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="K4" s="5" t="n">
         <v>4021827</v>
       </c>
-      <c r="K4" s="8" t="n">
+      <c r="L4" s="8" t="n">
         <v>2.72</v>
       </c>
-      <c r="L4" s="8" t="n">
+      <c r="M4" s="8" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="N4" s="8" t="n">
         <v>1.28</v>
       </c>
-      <c r="M4" s="8" t="n">
+      <c r="O4" s="8" t="n">
         <v>1.44</v>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>✅維持（7/26テスト判定）</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>61k+12k維持</t>
         </is>
@@ -1242,27 +1279,33 @@
       <c r="H5" s="11" t="n">
         <v>0.372</v>
       </c>
-      <c r="I5" s="10" t="n">
+      <c r="I5" s="12" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="J5" s="10" t="n">
         <v>156300</v>
       </c>
-      <c r="J5" s="10" t="n">
+      <c r="K5" s="10" t="n">
         <v>2316678</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>2.58</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="N5" s="12" t="n">
         <v>1.23</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="O5" s="12" t="n">
         <v>1.35</v>
       </c>
-      <c r="N5" s="9" t="inlineStr">
+      <c r="P5" s="9" t="inlineStr">
         <is>
           <t>✅BC検証中（7/25判定）</t>
         </is>
       </c>
-      <c r="O5" s="9" t="inlineStr">
+      <c r="Q5" s="9" t="inlineStr">
         <is>
           <t>50k+10k維持</t>
         </is>
@@ -1295,27 +1338,33 @@
       <c r="H6" s="6" t="n">
         <v>0.399</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="I6" s="8" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="J6" s="5" t="n">
         <v>145555</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="K6" s="5" t="n">
         <v>896586</v>
       </c>
-      <c r="K6" s="8" t="n">
+      <c r="L6" s="8" t="n">
         <v>3.35</v>
       </c>
-      <c r="L6" s="8" t="n">
+      <c r="M6" s="8" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="N6" s="8" t="n">
         <v>1.35</v>
       </c>
-      <c r="M6" s="8" t="n">
+      <c r="O6" s="8" t="n">
         <v>1.99</v>
       </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>✅41k好調（7/25判定）</t>
         </is>
       </c>
-      <c r="O6" s="4" t="inlineStr">
+      <c r="Q6" s="4" t="inlineStr">
         <is>
           <t>41k維持</t>
         </is>
@@ -1348,27 +1397,33 @@
       <c r="H7" s="11" t="n">
         <v>0.482</v>
       </c>
-      <c r="I7" s="10" t="n">
+      <c r="I7" s="12" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="J7" s="10" t="n">
         <v>175527</v>
       </c>
-      <c r="J7" s="10" t="n">
+      <c r="K7" s="10" t="n">
         <v>419751</v>
       </c>
-      <c r="K7" s="12" t="n">
+      <c r="L7" s="12" t="n">
         <v>4.63</v>
       </c>
-      <c r="L7" s="12" t="n">
+      <c r="M7" s="12" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="N7" s="12" t="n">
         <v>1.5</v>
       </c>
-      <c r="M7" s="12" t="n">
+      <c r="O7" s="12" t="n">
         <v>3.13</v>
       </c>
-      <c r="N7" s="9" t="inlineStr">
+      <c r="P7" s="9" t="inlineStr">
         <is>
           <t>✅30k好調（7/25判定）</t>
         </is>
       </c>
-      <c r="O7" s="9" t="inlineStr">
+      <c r="Q7" s="9" t="inlineStr">
         <is>
           <t>30k維持</t>
         </is>
@@ -1401,27 +1456,33 @@
       <c r="H8" s="6" t="n">
         <v>0.215</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="I8" s="8" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="J8" s="5" t="n">
         <v>64227</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="K8" s="5" t="n">
         <v>739765</v>
       </c>
-      <c r="K8" s="8" t="n">
+      <c r="L8" s="8" t="n">
         <v>2.74</v>
       </c>
-      <c r="L8" s="8" t="n">
+      <c r="M8" s="8" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="N8" s="8" t="n">
         <v>1.56</v>
       </c>
-      <c r="M8" s="8" t="n">
+      <c r="O8" s="8" t="n">
         <v>1.17</v>
       </c>
-      <c r="N8" s="4" t="inlineStr">
+      <c r="P8" s="4" t="inlineStr">
         <is>
           <t>✅34k好調（7/25判定）</t>
         </is>
       </c>
-      <c r="O8" s="4" t="inlineStr">
+      <c r="Q8" s="4" t="inlineStr">
         <is>
           <t>34k維持</t>
         </is>
@@ -1454,27 +1515,33 @@
       <c r="H9" s="11" t="n">
         <v>0.346</v>
       </c>
-      <c r="I9" s="10" t="n">
+      <c r="I9" s="12" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="J9" s="10" t="n">
         <v>66056</v>
       </c>
-      <c r="J9" s="10" t="n">
+      <c r="K9" s="10" t="n">
         <v>132224</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>5.59</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="N9" s="12" t="n">
         <v>1.59</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="O9" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="N9" s="9" t="inlineStr">
+      <c r="P9" s="9" t="inlineStr">
         <is>
           <t>🚀本日増額判定</t>
         </is>
       </c>
-      <c r="O9" s="9" t="inlineStr">
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>13k（7/25判定）</t>
         </is>
@@ -1507,27 +1574,33 @@
       <c r="H10" s="6" t="n">
         <v>0.233</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="I10" s="8" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="J10" s="5" t="n">
         <v>55629</v>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="K10" s="5" t="n">
         <v>235616</v>
       </c>
-      <c r="K10" s="8" t="n">
+      <c r="L10" s="8" t="n">
         <v>3.65</v>
       </c>
-      <c r="L10" s="8" t="n">
+      <c r="M10" s="8" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="N10" s="8" t="n">
         <v>1.72</v>
       </c>
-      <c r="M10" s="8" t="n">
+      <c r="O10" s="8" t="n">
         <v>1.93</v>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>✅16k好調（7/25判定）</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
+      <c r="Q10" s="4" t="inlineStr">
         <is>
           <t>16k維持</t>
         </is>
@@ -1560,27 +1633,33 @@
       <c r="H11" s="11" t="n">
         <v>0.33</v>
       </c>
-      <c r="I11" s="10" t="n">
+      <c r="I11" s="12" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="J11" s="10" t="n">
         <v>29344</v>
       </c>
-      <c r="J11" s="10" t="n">
+      <c r="K11" s="10" t="n">
         <v>375802</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>2.13</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="N11" s="12" t="n">
         <v>1.25</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="O11" s="12" t="n">
         <v>0.88</v>
       </c>
-      <c r="N11" s="9" t="inlineStr">
+      <c r="P11" s="9" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="O11" s="9" t="inlineStr">
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>17k維持</t>
         </is>
@@ -1613,27 +1692,33 @@
       <c r="H12" s="6" t="n">
         <v>0.157</v>
       </c>
-      <c r="I12" s="5" t="n">
+      <c r="I12" s="8" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="J12" s="5" t="n">
         <v>23504</v>
       </c>
-      <c r="J12" s="5" t="n">
+      <c r="K12" s="5" t="n">
         <v>553129</v>
       </c>
-      <c r="K12" s="8" t="n">
+      <c r="L12" s="8" t="n">
         <v>2.01</v>
       </c>
-      <c r="L12" s="8" t="n">
+      <c r="M12" s="8" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="N12" s="8" t="n">
         <v>1.33</v>
       </c>
-      <c r="M12" s="8" t="n">
+      <c r="O12" s="8" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="P12" s="4" t="inlineStr">
         <is>
           <t>⚠️先行指標点灯（CR/複製リセット準備）</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr">
+      <c r="Q12" s="4" t="inlineStr">
         <is>
           <t>22k維持</t>
         </is>
@@ -1666,27 +1751,33 @@
       <c r="H13" s="11" t="n">
         <v>0.477</v>
       </c>
-      <c r="I13" s="10" t="n">
+      <c r="I13" s="12" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="J13" s="10" t="n">
         <v>26879</v>
       </c>
-      <c r="J13" s="10" t="n">
+      <c r="K13" s="10" t="n">
         <v>306262</v>
       </c>
-      <c r="K13" s="12" t="n">
+      <c r="L13" s="12" t="n">
         <v>1.98</v>
       </c>
-      <c r="L13" s="12" t="n">
+      <c r="M13" s="12" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="N13" s="12" t="n">
         <v>1.31</v>
       </c>
-      <c r="M13" s="12" t="n">
+      <c r="O13" s="12" t="n">
         <v>0.67</v>
       </c>
-      <c r="N13" s="9" t="inlineStr">
+      <c r="P13" s="9" t="inlineStr">
         <is>
           <t>✅持ち直し</t>
         </is>
       </c>
-      <c r="O13" s="9" t="inlineStr">
+      <c r="Q13" s="9" t="inlineStr">
         <is>
           <t>13k維持</t>
         </is>
@@ -1719,21 +1810,23 @@
       <c r="H14" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I14" s="5" t="n">
+      <c r="I14" s="4" t="inlineStr"/>
+      <c r="J14" s="5" t="n">
         <v>21976</v>
       </c>
-      <c r="J14" s="5" t="n">
+      <c r="K14" s="5" t="n">
         <v>105592</v>
       </c>
-      <c r="K14" s="4" t="inlineStr"/>
       <c r="L14" s="4" t="inlineStr"/>
       <c r="M14" s="4" t="inlineStr"/>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr"/>
+      <c r="O14" s="4" t="inlineStr"/>
+      <c r="P14" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="O14" s="4" t="inlineStr">
+      <c r="Q14" s="4" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -1766,27 +1859,33 @@
       <c r="H15" s="11" t="n">
         <v>0.504</v>
       </c>
-      <c r="I15" s="10" t="n">
+      <c r="I15" s="12" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="J15" s="10" t="n">
         <v>24879</v>
       </c>
-      <c r="J15" s="10" t="n">
+      <c r="K15" s="10" t="n">
         <v>98342</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>1.76</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="N15" s="12" t="n">
         <v>1.34</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="O15" s="12" t="n">
         <v>0.41</v>
       </c>
-      <c r="N15" s="9" t="inlineStr">
+      <c r="P15" s="9" t="inlineStr">
         <is>
           <t>✅急回復・警戒解除</t>
         </is>
       </c>
-      <c r="O15" s="9" t="inlineStr">
+      <c r="Q15" s="9" t="inlineStr">
         <is>
           <t>13k維持</t>
         </is>
@@ -1819,21 +1918,23 @@
       <c r="H16" s="6" t="n">
         <v>0.646</v>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="5" t="n">
         <v>15444</v>
       </c>
-      <c r="J16" s="5" t="n">
+      <c r="K16" s="5" t="n">
         <v>69498</v>
       </c>
-      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="N16" s="4" t="inlineStr"/>
+      <c r="O16" s="4" t="inlineStr"/>
+      <c r="P16" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="O16" s="4" t="inlineStr">
+      <c r="Q16" s="4" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -1866,27 +1967,33 @@
       <c r="H17" s="11" t="n">
         <v>-0.062</v>
       </c>
-      <c r="I17" s="10" t="n">
+      <c r="I17" s="12" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="J17" s="10" t="n">
         <v>3816</v>
       </c>
-      <c r="J17" s="10" t="n">
+      <c r="K17" s="10" t="n">
         <v>221121</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>1.99</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="N17" s="12" t="n">
         <v>1.53</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="O17" s="12" t="n">
         <v>0.46</v>
       </c>
-      <c r="N17" s="9" t="inlineStr">
+      <c r="P17" s="9" t="inlineStr">
         <is>
           <t>✅監視</t>
         </is>
       </c>
-      <c r="O17" s="9" t="inlineStr">
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>11k維持</t>
         </is>
@@ -1919,27 +2026,33 @@
       <c r="H18" s="6" t="n">
         <v>-0.08799999999999999</v>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="I18" s="8" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="J18" s="5" t="n">
         <v>19354</v>
       </c>
-      <c r="J18" s="5" t="n">
+      <c r="K18" s="5" t="n">
         <v>43498</v>
       </c>
-      <c r="K18" s="8" t="n">
+      <c r="L18" s="8" t="n">
         <v>2.25</v>
       </c>
-      <c r="L18" s="8" t="n">
+      <c r="M18" s="8" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="N18" s="8" t="n">
         <v>1.88</v>
       </c>
-      <c r="M18" s="8" t="n">
+      <c r="O18" s="8" t="n">
         <v>0.37</v>
       </c>
-      <c r="N18" s="4" t="inlineStr">
+      <c r="P18" s="4" t="inlineStr">
         <is>
           <t>✅黒字維持（7/27判定）</t>
         </is>
       </c>
-      <c r="O18" s="4" t="inlineStr">
+      <c r="Q18" s="4" t="inlineStr">
         <is>
           <t>13k維持</t>
         </is>
@@ -1972,21 +2085,23 @@
       <c r="H19" s="11" t="n">
         <v>0.76</v>
       </c>
-      <c r="I19" s="10" t="n">
+      <c r="I19" s="9" t="inlineStr"/>
+      <c r="J19" s="10" t="n">
         <v>4545</v>
       </c>
-      <c r="J19" s="10" t="n">
+      <c r="K19" s="10" t="n">
         <v>40905</v>
       </c>
-      <c r="K19" s="9" t="inlineStr"/>
       <c r="L19" s="9" t="inlineStr"/>
       <c r="M19" s="9" t="inlineStr"/>
-      <c r="N19" s="9" t="inlineStr">
+      <c r="N19" s="9" t="inlineStr"/>
+      <c r="O19" s="9" t="inlineStr"/>
+      <c r="P19" s="9" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="O19" s="9" t="inlineStr">
+      <c r="Q19" s="9" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -2017,21 +2132,23 @@
         <v>0</v>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="5" t="n">
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J20" s="5" t="n">
+      <c r="K20" s="5" t="n">
         <v>6844</v>
       </c>
-      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" s="4" t="inlineStr">
+      <c r="N20" s="4" t="inlineStr"/>
+      <c r="O20" s="4" t="inlineStr"/>
+      <c r="P20" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="O20" s="4" t="inlineStr">
+      <c r="Q20" s="4" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -2062,21 +2179,23 @@
         <v>0</v>
       </c>
       <c r="H21" s="9" t="inlineStr"/>
-      <c r="I21" s="10" t="n">
+      <c r="I21" s="9" t="inlineStr"/>
+      <c r="J21" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="J21" s="10" t="n">
+      <c r="K21" s="10" t="n">
         <v>18235</v>
       </c>
-      <c r="K21" s="9" t="inlineStr"/>
       <c r="L21" s="9" t="inlineStr"/>
       <c r="M21" s="9" t="inlineStr"/>
-      <c r="N21" s="9" t="inlineStr">
+      <c r="N21" s="9" t="inlineStr"/>
+      <c r="O21" s="9" t="inlineStr"/>
+      <c r="P21" s="9" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="O21" s="9" t="inlineStr">
+      <c r="Q21" s="9" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -2109,27 +2228,33 @@
       <c r="H22" s="6" t="n">
         <v>-0.373</v>
       </c>
-      <c r="I22" s="5" t="n">
+      <c r="I22" s="8" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J22" s="5" t="n">
         <v>12423</v>
       </c>
-      <c r="J22" s="5" t="n">
+      <c r="K22" s="5" t="n">
         <v>112024</v>
       </c>
-      <c r="K22" s="8" t="n">
+      <c r="L22" s="8" t="n">
         <v>1.61</v>
       </c>
-      <c r="L22" s="8" t="n">
+      <c r="M22" s="8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N22" s="8" t="n">
         <v>1.58</v>
       </c>
-      <c r="M22" s="8" t="n">
+      <c r="O22" s="8" t="n">
         <v>0.03</v>
       </c>
-      <c r="N22" s="4" t="inlineStr">
+      <c r="P22" s="4" t="inlineStr">
         <is>
           <t>🔧段階②判定は7/26</t>
         </is>
       </c>
-      <c r="O22" s="4" t="inlineStr">
+      <c r="Q22" s="4" t="inlineStr">
         <is>
           <t>6.5k維持</t>
         </is>
@@ -2160,27 +2285,31 @@
         <v>-5232</v>
       </c>
       <c r="H23" s="9" t="inlineStr"/>
-      <c r="I23" s="10" t="n">
+      <c r="I23" s="9" t="inlineStr"/>
+      <c r="J23" s="10" t="n">
         <v>11097</v>
       </c>
-      <c r="J23" s="10" t="n">
+      <c r="K23" s="10" t="n">
         <v>104701</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>1.36</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="N23" s="12" t="n">
         <v>1.35</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="O23" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="N23" s="9" t="inlineStr">
+      <c r="P23" s="9" t="inlineStr">
         <is>
           <t>🔧CRシェア58%獲得（7/29判定）</t>
         </is>
       </c>
-      <c r="O23" s="9" t="inlineStr">
+      <c r="Q23" s="9" t="inlineStr">
         <is>
           <t>5k維持</t>
         </is>
@@ -2213,27 +2342,33 @@
       <c r="H24" s="6" t="n">
         <v>-0.016</v>
       </c>
-      <c r="I24" s="14" t="n">
+      <c r="I24" s="8" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J24" s="14" t="n">
         <v>-14886</v>
       </c>
-      <c r="J24" s="5" t="n">
+      <c r="K24" s="5" t="n">
         <v>130758</v>
       </c>
-      <c r="K24" s="8" t="n">
+      <c r="L24" s="8" t="n">
         <v>1.42</v>
       </c>
-      <c r="L24" s="8" t="n">
+      <c r="M24" s="8" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="N24" s="8" t="n">
         <v>1.51</v>
       </c>
-      <c r="M24" s="8" t="n">
+      <c r="O24" s="8" t="n">
         <v>-0.08</v>
       </c>
-      <c r="N24" s="4" t="inlineStr">
+      <c r="P24" s="4" t="inlineStr">
         <is>
           <t>🔧全開放テスト中（8/6判定）</t>
         </is>
       </c>
-      <c r="O24" s="4" t="inlineStr">
+      <c r="Q24" s="4" t="inlineStr">
         <is>
           <t>6k+6k維持</t>
         </is>
@@ -2266,27 +2401,33 @@
       <c r="H25" s="11" t="n">
         <v>-0.6879999999999999</v>
       </c>
-      <c r="I25" s="13" t="n">
+      <c r="I25" s="12" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J25" s="13" t="n">
         <v>-18790</v>
       </c>
-      <c r="J25" s="10" t="n">
+      <c r="K25" s="10" t="n">
         <v>222657</v>
       </c>
-      <c r="K25" s="12" t="n">
+      <c r="L25" s="12" t="n">
         <v>1.41</v>
       </c>
-      <c r="L25" s="12" t="n">
+      <c r="M25" s="12" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="N25" s="12" t="n">
         <v>1.63</v>
       </c>
-      <c r="M25" s="12" t="n">
+      <c r="O25" s="12" t="n">
         <v>-0.22</v>
       </c>
-      <c r="N25" s="9" t="inlineStr">
+      <c r="P25" s="9" t="inlineStr">
         <is>
           <t>🔧複製リセット中（7/30判定）</t>
         </is>
       </c>
-      <c r="O25" s="9" t="inlineStr">
+      <c r="Q25" s="9" t="inlineStr">
         <is>
           <t>10k維持</t>
         </is>
@@ -2317,21 +2458,23 @@
         <v>0</v>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="5" t="n">
+      <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J26" s="5" t="n">
+      <c r="K26" s="5" t="n">
         <v>55764</v>
       </c>
-      <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="4" t="inlineStr"/>
       <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" s="4" t="inlineStr">
+      <c r="N26" s="4" t="inlineStr"/>
+      <c r="O26" s="4" t="inlineStr"/>
+      <c r="P26" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="O26" s="4" t="inlineStr">
+      <c r="Q26" s="4" t="inlineStr">
         <is>
           <t>−</t>
         </is>

</xml_diff>

<commit_message>
Remove ROAS columns per user decision; MER remains the decision metric
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-07-24.xlsx
+++ b/data/reports/report-2026-07-24.xlsx
@@ -951,7 +951,7 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>・MER(7日)=Shopify売上(7日)÷Meta広告費(7日)。ROAS=Meta計上コンバージョン価値÷広告費（手計算値・Meta表示列は不使用）。前日ROASは単日値のためブレが大きく参考値</t>
+          <t>・MER(7日)=Shopify売上(7日)÷Meta広告費(7日)＝実売ベースの広告効率（意思決定はこの指標）。ROAS列は2026-07-24ユーザー判断で廃止（Meta計上値は突合チェックと広告セット/CR単位の判定にのみ内部使用）</t>
         </is>
       </c>
     </row>
@@ -966,7 +966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q26"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -977,15 +977,13 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="7" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1031,45 +1029,35 @@
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>前日ROAS</t>
+          <t>3日利益</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
-          <t>3日利益</t>
+          <t>30日利益</t>
         </is>
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
-          <t>30日利益</t>
+          <t>MER(7日)</t>
         </is>
       </c>
       <c r="L1" s="3" t="inlineStr">
         <is>
-          <t>MER(7日)</t>
+          <t>分岐</t>
         </is>
       </c>
       <c r="M1" s="3" t="inlineStr">
         <is>
-          <t>ROAS(7日)</t>
+          <t>余裕</t>
         </is>
       </c>
       <c r="N1" s="3" t="inlineStr">
         <is>
-          <t>分岐</t>
+          <t>判定</t>
         </is>
       </c>
       <c r="O1" s="3" t="inlineStr">
-        <is>
-          <t>余裕</t>
-        </is>
-      </c>
-      <c r="P1" s="3" t="inlineStr">
-        <is>
-          <t>判定</t>
-        </is>
-      </c>
-      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>予算</t>
         </is>
@@ -1102,33 +1090,27 @@
       <c r="H2" s="6" t="n">
         <v>0.435</v>
       </c>
-      <c r="I2" s="8" t="n">
-        <v>3.51</v>
+      <c r="I2" s="5" t="n">
+        <v>455982</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>455982</v>
-      </c>
-      <c r="K2" s="5" t="n">
         <v>2613247</v>
       </c>
+      <c r="K2" s="8" t="n">
+        <v>4.36</v>
+      </c>
       <c r="L2" s="8" t="n">
-        <v>4.36</v>
+        <v>1.53</v>
       </c>
       <c r="M2" s="8" t="n">
-        <v>3.42</v>
-      </c>
-      <c r="N2" s="8" t="n">
-        <v>1.53</v>
-      </c>
-      <c r="O2" s="8" t="n">
         <v>2.82</v>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>🎉記録更新（本日7/25判定）</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>85k維持</t>
         </is>
@@ -1161,33 +1143,27 @@
       <c r="H3" s="11" t="n">
         <v>0.357</v>
       </c>
-      <c r="I3" s="12" t="n">
-        <v>2.82</v>
+      <c r="I3" s="10" t="n">
+        <v>311271</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>311271</v>
-      </c>
-      <c r="K3" s="10" t="n">
         <v>2036918</v>
       </c>
+      <c r="K3" s="12" t="n">
+        <v>3.24</v>
+      </c>
       <c r="L3" s="12" t="n">
-        <v>3.24</v>
+        <v>1.35</v>
       </c>
       <c r="M3" s="12" t="n">
-        <v>2.92</v>
-      </c>
-      <c r="N3" s="12" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="O3" s="12" t="n">
         <v>1.88</v>
       </c>
-      <c r="P3" s="9" t="inlineStr">
+      <c r="N3" s="9" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
+      <c r="O3" s="9" t="inlineStr">
         <is>
           <t>35k+25k維持</t>
         </is>
@@ -1220,33 +1196,27 @@
       <c r="H4" s="6" t="n">
         <v>0.356</v>
       </c>
-      <c r="I4" s="8" t="n">
-        <v>1.95</v>
+      <c r="I4" s="5" t="n">
+        <v>218426</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>218426</v>
-      </c>
-      <c r="K4" s="5" t="n">
         <v>4021827</v>
       </c>
+      <c r="K4" s="8" t="n">
+        <v>2.72</v>
+      </c>
       <c r="L4" s="8" t="n">
-        <v>2.72</v>
+        <v>1.28</v>
       </c>
       <c r="M4" s="8" t="n">
-        <v>2.14</v>
-      </c>
-      <c r="N4" s="8" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="O4" s="8" t="n">
         <v>1.44</v>
       </c>
-      <c r="P4" s="4" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>✅維持（7/26テスト判定）</t>
         </is>
       </c>
-      <c r="Q4" s="4" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>61k+12k維持</t>
         </is>
@@ -1279,33 +1249,27 @@
       <c r="H5" s="11" t="n">
         <v>0.372</v>
       </c>
-      <c r="I5" s="12" t="n">
-        <v>1.76</v>
+      <c r="I5" s="10" t="n">
+        <v>156300</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>156300</v>
-      </c>
-      <c r="K5" s="10" t="n">
         <v>2316678</v>
       </c>
+      <c r="K5" s="12" t="n">
+        <v>2.58</v>
+      </c>
       <c r="L5" s="12" t="n">
-        <v>2.58</v>
+        <v>1.23</v>
       </c>
       <c r="M5" s="12" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>1.23</v>
-      </c>
-      <c r="O5" s="12" t="n">
         <v>1.35</v>
       </c>
-      <c r="P5" s="9" t="inlineStr">
+      <c r="N5" s="9" t="inlineStr">
         <is>
           <t>✅BC検証中（7/25判定）</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
+      <c r="O5" s="9" t="inlineStr">
         <is>
           <t>50k+10k維持</t>
         </is>
@@ -1338,33 +1302,27 @@
       <c r="H6" s="6" t="n">
         <v>0.399</v>
       </c>
-      <c r="I6" s="8" t="n">
-        <v>2.82</v>
+      <c r="I6" s="5" t="n">
+        <v>145555</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>145555</v>
-      </c>
-      <c r="K6" s="5" t="n">
         <v>896586</v>
       </c>
+      <c r="K6" s="8" t="n">
+        <v>3.35</v>
+      </c>
       <c r="L6" s="8" t="n">
-        <v>3.35</v>
+        <v>1.35</v>
       </c>
       <c r="M6" s="8" t="n">
-        <v>3.02</v>
-      </c>
-      <c r="N6" s="8" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="O6" s="8" t="n">
         <v>1.99</v>
       </c>
-      <c r="P6" s="4" t="inlineStr">
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>✅41k好調（7/25判定）</t>
         </is>
       </c>
-      <c r="Q6" s="4" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>41k維持</t>
         </is>
@@ -1397,33 +1355,27 @@
       <c r="H7" s="11" t="n">
         <v>0.482</v>
       </c>
-      <c r="I7" s="12" t="n">
-        <v>3.58</v>
+      <c r="I7" s="10" t="n">
+        <v>175527</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>175527</v>
-      </c>
-      <c r="K7" s="10" t="n">
         <v>419751</v>
       </c>
+      <c r="K7" s="12" t="n">
+        <v>4.63</v>
+      </c>
       <c r="L7" s="12" t="n">
-        <v>4.63</v>
+        <v>1.5</v>
       </c>
       <c r="M7" s="12" t="n">
-        <v>3.93</v>
-      </c>
-      <c r="N7" s="12" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="O7" s="12" t="n">
         <v>3.13</v>
       </c>
-      <c r="P7" s="9" t="inlineStr">
+      <c r="N7" s="9" t="inlineStr">
         <is>
           <t>✅30k好調（7/25判定）</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
+      <c r="O7" s="9" t="inlineStr">
         <is>
           <t>30k維持</t>
         </is>
@@ -1456,33 +1408,27 @@
       <c r="H8" s="6" t="n">
         <v>0.215</v>
       </c>
-      <c r="I8" s="8" t="n">
-        <v>2.08</v>
+      <c r="I8" s="5" t="n">
+        <v>64227</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>64227</v>
-      </c>
-      <c r="K8" s="5" t="n">
         <v>739765</v>
       </c>
+      <c r="K8" s="8" t="n">
+        <v>2.74</v>
+      </c>
       <c r="L8" s="8" t="n">
-        <v>2.74</v>
+        <v>1.56</v>
       </c>
       <c r="M8" s="8" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="N8" s="8" t="n">
-        <v>1.56</v>
-      </c>
-      <c r="O8" s="8" t="n">
         <v>1.17</v>
       </c>
-      <c r="P8" s="4" t="inlineStr">
+      <c r="N8" s="4" t="inlineStr">
         <is>
           <t>✅34k好調（7/25判定）</t>
         </is>
       </c>
-      <c r="Q8" s="4" t="inlineStr">
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>34k維持</t>
         </is>
@@ -1515,33 +1461,27 @@
       <c r="H9" s="11" t="n">
         <v>0.346</v>
       </c>
-      <c r="I9" s="12" t="n">
-        <v>3.43</v>
+      <c r="I9" s="10" t="n">
+        <v>66056</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>66056</v>
-      </c>
-      <c r="K9" s="10" t="n">
         <v>132224</v>
       </c>
+      <c r="K9" s="12" t="n">
+        <v>5.59</v>
+      </c>
       <c r="L9" s="12" t="n">
-        <v>5.59</v>
+        <v>1.59</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>5.25</v>
-      </c>
-      <c r="N9" s="12" t="n">
-        <v>1.59</v>
-      </c>
-      <c r="O9" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="P9" s="9" t="inlineStr">
+      <c r="N9" s="9" t="inlineStr">
         <is>
           <t>🚀本日増額判定</t>
         </is>
       </c>
-      <c r="Q9" s="9" t="inlineStr">
+      <c r="O9" s="9" t="inlineStr">
         <is>
           <t>13k（7/25判定）</t>
         </is>
@@ -1574,33 +1514,27 @@
       <c r="H10" s="6" t="n">
         <v>0.233</v>
       </c>
-      <c r="I10" s="8" t="n">
-        <v>1.64</v>
+      <c r="I10" s="5" t="n">
+        <v>55629</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>55629</v>
-      </c>
-      <c r="K10" s="5" t="n">
         <v>235616</v>
       </c>
+      <c r="K10" s="8" t="n">
+        <v>3.65</v>
+      </c>
       <c r="L10" s="8" t="n">
-        <v>3.65</v>
+        <v>1.72</v>
       </c>
       <c r="M10" s="8" t="n">
-        <v>2.68</v>
-      </c>
-      <c r="N10" s="8" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="O10" s="8" t="n">
         <v>1.93</v>
       </c>
-      <c r="P10" s="4" t="inlineStr">
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>✅16k好調（7/25判定）</t>
         </is>
       </c>
-      <c r="Q10" s="4" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>16k維持</t>
         </is>
@@ -1633,33 +1567,27 @@
       <c r="H11" s="11" t="n">
         <v>0.33</v>
       </c>
-      <c r="I11" s="12" t="n">
-        <v>1.56</v>
+      <c r="I11" s="10" t="n">
+        <v>29344</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>29344</v>
-      </c>
-      <c r="K11" s="10" t="n">
         <v>375802</v>
       </c>
+      <c r="K11" s="12" t="n">
+        <v>2.13</v>
+      </c>
       <c r="L11" s="12" t="n">
-        <v>2.13</v>
+        <v>1.25</v>
       </c>
       <c r="M11" s="12" t="n">
-        <v>1.84</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="O11" s="12" t="n">
         <v>0.88</v>
       </c>
-      <c r="P11" s="9" t="inlineStr">
+      <c r="N11" s="9" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
+      <c r="O11" s="9" t="inlineStr">
         <is>
           <t>17k維持</t>
         </is>
@@ -1692,33 +1620,27 @@
       <c r="H12" s="6" t="n">
         <v>0.157</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>1.66</v>
+      <c r="I12" s="5" t="n">
+        <v>23504</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>23504</v>
-      </c>
-      <c r="K12" s="5" t="n">
         <v>553129</v>
       </c>
+      <c r="K12" s="8" t="n">
+        <v>2.01</v>
+      </c>
       <c r="L12" s="8" t="n">
-        <v>2.01</v>
+        <v>1.33</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="O12" s="8" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="P12" s="4" t="inlineStr">
+      <c r="N12" s="4" t="inlineStr">
         <is>
           <t>⚠️先行指標点灯（CR/複製リセット準備）</t>
         </is>
       </c>
-      <c r="Q12" s="4" t="inlineStr">
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>22k維持</t>
         </is>
@@ -1751,33 +1673,27 @@
       <c r="H13" s="11" t="n">
         <v>0.477</v>
       </c>
-      <c r="I13" s="12" t="n">
-        <v>2.85</v>
+      <c r="I13" s="10" t="n">
+        <v>26879</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>26879</v>
-      </c>
-      <c r="K13" s="10" t="n">
         <v>306262</v>
       </c>
+      <c r="K13" s="12" t="n">
+        <v>1.98</v>
+      </c>
       <c r="L13" s="12" t="n">
-        <v>1.98</v>
+        <v>1.31</v>
       </c>
       <c r="M13" s="12" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="N13" s="12" t="n">
-        <v>1.31</v>
-      </c>
-      <c r="O13" s="12" t="n">
         <v>0.67</v>
       </c>
-      <c r="P13" s="9" t="inlineStr">
+      <c r="N13" s="9" t="inlineStr">
         <is>
           <t>✅持ち直し</t>
         </is>
       </c>
-      <c r="Q13" s="9" t="inlineStr">
+      <c r="O13" s="9" t="inlineStr">
         <is>
           <t>13k維持</t>
         </is>
@@ -1810,23 +1726,21 @@
       <c r="H14" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I14" s="4" t="inlineStr"/>
+      <c r="I14" s="5" t="n">
+        <v>21976</v>
+      </c>
       <c r="J14" s="5" t="n">
-        <v>21976</v>
-      </c>
-      <c r="K14" s="5" t="n">
         <v>105592</v>
       </c>
+      <c r="K14" s="4" t="inlineStr"/>
       <c r="L14" s="4" t="inlineStr"/>
       <c r="M14" s="4" t="inlineStr"/>
-      <c r="N14" s="4" t="inlineStr"/>
-      <c r="O14" s="4" t="inlineStr"/>
-      <c r="P14" s="4" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="Q14" s="4" t="inlineStr">
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -1859,33 +1773,27 @@
       <c r="H15" s="11" t="n">
         <v>0.504</v>
       </c>
-      <c r="I15" s="12" t="n">
-        <v>3.91</v>
+      <c r="I15" s="10" t="n">
+        <v>24879</v>
       </c>
       <c r="J15" s="10" t="n">
-        <v>24879</v>
-      </c>
-      <c r="K15" s="10" t="n">
         <v>98342</v>
       </c>
+      <c r="K15" s="12" t="n">
+        <v>1.76</v>
+      </c>
       <c r="L15" s="12" t="n">
-        <v>1.76</v>
+        <v>1.34</v>
       </c>
       <c r="M15" s="12" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="N15" s="12" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="O15" s="12" t="n">
         <v>0.41</v>
       </c>
-      <c r="P15" s="9" t="inlineStr">
+      <c r="N15" s="9" t="inlineStr">
         <is>
           <t>✅急回復・警戒解除</t>
         </is>
       </c>
-      <c r="Q15" s="9" t="inlineStr">
+      <c r="O15" s="9" t="inlineStr">
         <is>
           <t>13k維持</t>
         </is>
@@ -1918,23 +1826,21 @@
       <c r="H16" s="6" t="n">
         <v>0.646</v>
       </c>
-      <c r="I16" s="4" t="inlineStr"/>
+      <c r="I16" s="5" t="n">
+        <v>15444</v>
+      </c>
       <c r="J16" s="5" t="n">
-        <v>15444</v>
-      </c>
-      <c r="K16" s="5" t="n">
         <v>69498</v>
       </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr"/>
-      <c r="O16" s="4" t="inlineStr"/>
-      <c r="P16" s="4" t="inlineStr">
+      <c r="N16" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="Q16" s="4" t="inlineStr">
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -1967,33 +1873,27 @@
       <c r="H17" s="11" t="n">
         <v>-0.062</v>
       </c>
-      <c r="I17" s="12" t="n">
-        <v>1.42</v>
+      <c r="I17" s="10" t="n">
+        <v>3816</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>3816</v>
-      </c>
-      <c r="K17" s="10" t="n">
         <v>221121</v>
       </c>
+      <c r="K17" s="12" t="n">
+        <v>1.99</v>
+      </c>
       <c r="L17" s="12" t="n">
-        <v>1.99</v>
+        <v>1.53</v>
       </c>
       <c r="M17" s="12" t="n">
-        <v>1.89</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>1.53</v>
-      </c>
-      <c r="O17" s="12" t="n">
         <v>0.46</v>
       </c>
-      <c r="P17" s="9" t="inlineStr">
+      <c r="N17" s="9" t="inlineStr">
         <is>
           <t>✅監視</t>
         </is>
       </c>
-      <c r="Q17" s="9" t="inlineStr">
+      <c r="O17" s="9" t="inlineStr">
         <is>
           <t>11k維持</t>
         </is>
@@ -2026,33 +1926,27 @@
       <c r="H18" s="6" t="n">
         <v>-0.08799999999999999</v>
       </c>
-      <c r="I18" s="8" t="n">
-        <v>1.61</v>
+      <c r="I18" s="5" t="n">
+        <v>19354</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>19354</v>
-      </c>
-      <c r="K18" s="5" t="n">
         <v>43498</v>
       </c>
+      <c r="K18" s="8" t="n">
+        <v>2.25</v>
+      </c>
       <c r="L18" s="8" t="n">
-        <v>2.25</v>
+        <v>1.88</v>
       </c>
       <c r="M18" s="8" t="n">
-        <v>2.14</v>
-      </c>
-      <c r="N18" s="8" t="n">
-        <v>1.88</v>
-      </c>
-      <c r="O18" s="8" t="n">
         <v>0.37</v>
       </c>
-      <c r="P18" s="4" t="inlineStr">
+      <c r="N18" s="4" t="inlineStr">
         <is>
           <t>✅黒字維持（7/27判定）</t>
         </is>
       </c>
-      <c r="Q18" s="4" t="inlineStr">
+      <c r="O18" s="4" t="inlineStr">
         <is>
           <t>13k維持</t>
         </is>
@@ -2085,23 +1979,21 @@
       <c r="H19" s="11" t="n">
         <v>0.76</v>
       </c>
-      <c r="I19" s="9" t="inlineStr"/>
+      <c r="I19" s="10" t="n">
+        <v>4545</v>
+      </c>
       <c r="J19" s="10" t="n">
-        <v>4545</v>
-      </c>
-      <c r="K19" s="10" t="n">
         <v>40905</v>
       </c>
+      <c r="K19" s="9" t="inlineStr"/>
       <c r="L19" s="9" t="inlineStr"/>
       <c r="M19" s="9" t="inlineStr"/>
-      <c r="N19" s="9" t="inlineStr"/>
-      <c r="O19" s="9" t="inlineStr"/>
-      <c r="P19" s="9" t="inlineStr">
+      <c r="N19" s="9" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="Q19" s="9" t="inlineStr">
+      <c r="O19" s="9" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -2132,23 +2024,21 @@
         <v>0</v>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="4" t="inlineStr"/>
+      <c r="I20" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="J20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" s="5" t="n">
         <v>6844</v>
       </c>
+      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" s="4" t="inlineStr"/>
-      <c r="O20" s="4" t="inlineStr"/>
-      <c r="P20" s="4" t="inlineStr">
+      <c r="N20" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="Q20" s="4" t="inlineStr">
+      <c r="O20" s="4" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -2179,23 +2069,21 @@
         <v>0</v>
       </c>
       <c r="H21" s="9" t="inlineStr"/>
-      <c r="I21" s="9" t="inlineStr"/>
+      <c r="I21" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="J21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="10" t="n">
         <v>18235</v>
       </c>
+      <c r="K21" s="9" t="inlineStr"/>
       <c r="L21" s="9" t="inlineStr"/>
       <c r="M21" s="9" t="inlineStr"/>
-      <c r="N21" s="9" t="inlineStr"/>
-      <c r="O21" s="9" t="inlineStr"/>
-      <c r="P21" s="9" t="inlineStr">
+      <c r="N21" s="9" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="Q21" s="9" t="inlineStr">
+      <c r="O21" s="9" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -2228,33 +2116,27 @@
       <c r="H22" s="6" t="n">
         <v>-0.373</v>
       </c>
-      <c r="I22" s="8" t="n">
-        <v>0.97</v>
+      <c r="I22" s="5" t="n">
+        <v>12423</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>12423</v>
-      </c>
-      <c r="K22" s="5" t="n">
         <v>112024</v>
       </c>
+      <c r="K22" s="8" t="n">
+        <v>1.61</v>
+      </c>
       <c r="L22" s="8" t="n">
-        <v>1.61</v>
+        <v>1.58</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="N22" s="8" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="O22" s="8" t="n">
         <v>0.03</v>
       </c>
-      <c r="P22" s="4" t="inlineStr">
+      <c r="N22" s="4" t="inlineStr">
         <is>
           <t>🔧段階②判定は7/26</t>
         </is>
       </c>
-      <c r="Q22" s="4" t="inlineStr">
+      <c r="O22" s="4" t="inlineStr">
         <is>
           <t>6.5k維持</t>
         </is>
@@ -2285,31 +2167,27 @@
         <v>-5232</v>
       </c>
       <c r="H23" s="9" t="inlineStr"/>
-      <c r="I23" s="9" t="inlineStr"/>
+      <c r="I23" s="10" t="n">
+        <v>11097</v>
+      </c>
       <c r="J23" s="10" t="n">
-        <v>11097</v>
-      </c>
-      <c r="K23" s="10" t="n">
         <v>104701</v>
       </c>
+      <c r="K23" s="12" t="n">
+        <v>1.36</v>
+      </c>
       <c r="L23" s="12" t="n">
-        <v>1.36</v>
+        <v>1.35</v>
       </c>
       <c r="M23" s="12" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="N23" s="12" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="O23" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="9" t="inlineStr">
+      <c r="N23" s="9" t="inlineStr">
         <is>
           <t>🔧CRシェア58%獲得（7/29判定）</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
+      <c r="O23" s="9" t="inlineStr">
         <is>
           <t>5k維持</t>
         </is>
@@ -2342,33 +2220,27 @@
       <c r="H24" s="6" t="n">
         <v>-0.016</v>
       </c>
-      <c r="I24" s="8" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="J24" s="14" t="n">
+      <c r="I24" s="14" t="n">
         <v>-14886</v>
       </c>
-      <c r="K24" s="5" t="n">
+      <c r="J24" s="5" t="n">
         <v>130758</v>
       </c>
+      <c r="K24" s="8" t="n">
+        <v>1.42</v>
+      </c>
       <c r="L24" s="8" t="n">
-        <v>1.42</v>
+        <v>1.51</v>
       </c>
       <c r="M24" s="8" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="N24" s="8" t="n">
-        <v>1.51</v>
-      </c>
-      <c r="O24" s="8" t="n">
         <v>-0.08</v>
       </c>
-      <c r="P24" s="4" t="inlineStr">
+      <c r="N24" s="4" t="inlineStr">
         <is>
           <t>🔧全開放テスト中（8/6判定）</t>
         </is>
       </c>
-      <c r="Q24" s="4" t="inlineStr">
+      <c r="O24" s="4" t="inlineStr">
         <is>
           <t>6k+6k維持</t>
         </is>
@@ -2401,33 +2273,27 @@
       <c r="H25" s="11" t="n">
         <v>-0.6879999999999999</v>
       </c>
-      <c r="I25" s="12" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="J25" s="13" t="n">
+      <c r="I25" s="13" t="n">
         <v>-18790</v>
       </c>
-      <c r="K25" s="10" t="n">
+      <c r="J25" s="10" t="n">
         <v>222657</v>
       </c>
+      <c r="K25" s="12" t="n">
+        <v>1.41</v>
+      </c>
       <c r="L25" s="12" t="n">
-        <v>1.41</v>
+        <v>1.63</v>
       </c>
       <c r="M25" s="12" t="n">
-        <v>1.39</v>
-      </c>
-      <c r="N25" s="12" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="O25" s="12" t="n">
         <v>-0.22</v>
       </c>
-      <c r="P25" s="9" t="inlineStr">
+      <c r="N25" s="9" t="inlineStr">
         <is>
           <t>🔧複製リセット中（7/30判定）</t>
         </is>
       </c>
-      <c r="Q25" s="9" t="inlineStr">
+      <c r="O25" s="9" t="inlineStr">
         <is>
           <t>10k維持</t>
         </is>
@@ -2458,23 +2324,21 @@
         <v>0</v>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="4" t="inlineStr"/>
+      <c r="I26" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="J26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" s="5" t="n">
         <v>55764</v>
       </c>
+      <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="4" t="inlineStr"/>
       <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" s="4" t="inlineStr"/>
-      <c r="O26" s="4" t="inlineStr"/>
-      <c r="P26" s="4" t="inlineStr">
+      <c r="N26" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="Q26" s="4" t="inlineStr">
+      <c r="O26" s="4" t="inlineStr">
         <is>
           <t>−</t>
         </is>

</xml_diff>

<commit_message>
Add current daily budget column to Excel product sheet
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-07-24.xlsx
+++ b/data/reports/report-2026-07-24.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -955,6 +955,13 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>・現日予算はセット合算（形状記憶=本体35k+テスト25k、害虫=本体61k+テスト12k、ナノガラス=本体50k+BC検証10k、ディスペンサー=類似6k+全開放6k）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -966,7 +973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -982,8 +989,9 @@
     <col width="8" customWidth="1" min="11" max="11"/>
     <col width="7" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1054,12 +1062,17 @@
       </c>
       <c r="N1" s="3" t="inlineStr">
         <is>
+          <t>現日予算(円)</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
           <t>判定</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
-        <is>
-          <t>予算</t>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>予算提案</t>
         </is>
       </c>
     </row>
@@ -1105,12 +1118,15 @@
       <c r="M2" s="8" t="n">
         <v>2.82</v>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="N2" s="5" t="n">
+        <v>85000</v>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>🎉記録更新（本日7/25判定）</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>85k維持</t>
         </is>
@@ -1158,12 +1174,15 @@
       <c r="M3" s="12" t="n">
         <v>1.88</v>
       </c>
-      <c r="N3" s="9" t="inlineStr">
+      <c r="N3" s="10" t="n">
+        <v>60000</v>
+      </c>
+      <c r="O3" s="9" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="O3" s="9" t="inlineStr">
+      <c r="P3" s="9" t="inlineStr">
         <is>
           <t>35k+25k維持</t>
         </is>
@@ -1211,12 +1230,15 @@
       <c r="M4" s="8" t="n">
         <v>1.44</v>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N4" s="5" t="n">
+        <v>73000</v>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>✅維持（7/26テスト判定）</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>61k+12k維持</t>
         </is>
@@ -1264,12 +1286,15 @@
       <c r="M5" s="12" t="n">
         <v>1.35</v>
       </c>
-      <c r="N5" s="9" t="inlineStr">
+      <c r="N5" s="10" t="n">
+        <v>60000</v>
+      </c>
+      <c r="O5" s="9" t="inlineStr">
         <is>
           <t>✅BC検証中（7/25判定）</t>
         </is>
       </c>
-      <c r="O5" s="9" t="inlineStr">
+      <c r="P5" s="9" t="inlineStr">
         <is>
           <t>50k+10k維持</t>
         </is>
@@ -1317,12 +1342,15 @@
       <c r="M6" s="8" t="n">
         <v>1.99</v>
       </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="N6" s="5" t="n">
+        <v>41000</v>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>✅41k好調（7/25判定）</t>
         </is>
       </c>
-      <c r="O6" s="4" t="inlineStr">
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>41k維持</t>
         </is>
@@ -1370,12 +1398,15 @@
       <c r="M7" s="12" t="n">
         <v>3.13</v>
       </c>
-      <c r="N7" s="9" t="inlineStr">
+      <c r="N7" s="10" t="n">
+        <v>30000</v>
+      </c>
+      <c r="O7" s="9" t="inlineStr">
         <is>
           <t>✅30k好調（7/25判定）</t>
         </is>
       </c>
-      <c r="O7" s="9" t="inlineStr">
+      <c r="P7" s="9" t="inlineStr">
         <is>
           <t>30k維持</t>
         </is>
@@ -1423,12 +1454,15 @@
       <c r="M8" s="8" t="n">
         <v>1.17</v>
       </c>
-      <c r="N8" s="4" t="inlineStr">
+      <c r="N8" s="5" t="n">
+        <v>34000</v>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>✅34k好調（7/25判定）</t>
         </is>
       </c>
-      <c r="O8" s="4" t="inlineStr">
+      <c r="P8" s="4" t="inlineStr">
         <is>
           <t>34k維持</t>
         </is>
@@ -1476,12 +1510,15 @@
       <c r="M9" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="N9" s="9" t="inlineStr">
+      <c r="N9" s="10" t="n">
+        <v>13000</v>
+      </c>
+      <c r="O9" s="9" t="inlineStr">
         <is>
           <t>🚀本日増額判定</t>
         </is>
       </c>
-      <c r="O9" s="9" t="inlineStr">
+      <c r="P9" s="9" t="inlineStr">
         <is>
           <t>13k（7/25判定）</t>
         </is>
@@ -1529,12 +1566,15 @@
       <c r="M10" s="8" t="n">
         <v>1.93</v>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="N10" s="5" t="n">
+        <v>16000</v>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>✅16k好調（7/25判定）</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>16k維持</t>
         </is>
@@ -1582,12 +1622,15 @@
       <c r="M11" s="12" t="n">
         <v>0.88</v>
       </c>
-      <c r="N11" s="9" t="inlineStr">
+      <c r="N11" s="10" t="n">
+        <v>17000</v>
+      </c>
+      <c r="O11" s="9" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="O11" s="9" t="inlineStr">
+      <c r="P11" s="9" t="inlineStr">
         <is>
           <t>17k維持</t>
         </is>
@@ -1635,12 +1678,15 @@
       <c r="M12" s="8" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="N12" s="5" t="n">
+        <v>22000</v>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>⚠️先行指標点灯（CR/複製リセット準備）</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr">
+      <c r="P12" s="4" t="inlineStr">
         <is>
           <t>22k維持</t>
         </is>
@@ -1688,12 +1734,15 @@
       <c r="M13" s="12" t="n">
         <v>0.67</v>
       </c>
-      <c r="N13" s="9" t="inlineStr">
+      <c r="N13" s="10" t="n">
+        <v>13000</v>
+      </c>
+      <c r="O13" s="9" t="inlineStr">
         <is>
           <t>✅持ち直し</t>
         </is>
       </c>
-      <c r="O13" s="9" t="inlineStr">
+      <c r="P13" s="9" t="inlineStr">
         <is>
           <t>13k維持</t>
         </is>
@@ -1735,12 +1784,13 @@
       <c r="K14" s="4" t="inlineStr"/>
       <c r="L14" s="4" t="inlineStr"/>
       <c r="M14" s="4" t="inlineStr"/>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr"/>
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="O14" s="4" t="inlineStr">
+      <c r="P14" s="4" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -1788,12 +1838,15 @@
       <c r="M15" s="12" t="n">
         <v>0.41</v>
       </c>
-      <c r="N15" s="9" t="inlineStr">
+      <c r="N15" s="10" t="n">
+        <v>13000</v>
+      </c>
+      <c r="O15" s="9" t="inlineStr">
         <is>
           <t>✅急回復・警戒解除</t>
         </is>
       </c>
-      <c r="O15" s="9" t="inlineStr">
+      <c r="P15" s="9" t="inlineStr">
         <is>
           <t>13k維持</t>
         </is>
@@ -1835,12 +1888,13 @@
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="N16" s="4" t="inlineStr"/>
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="O16" s="4" t="inlineStr">
+      <c r="P16" s="4" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -1888,12 +1942,15 @@
       <c r="M17" s="12" t="n">
         <v>0.46</v>
       </c>
-      <c r="N17" s="9" t="inlineStr">
+      <c r="N17" s="10" t="n">
+        <v>11000</v>
+      </c>
+      <c r="O17" s="9" t="inlineStr">
         <is>
           <t>✅監視</t>
         </is>
       </c>
-      <c r="O17" s="9" t="inlineStr">
+      <c r="P17" s="9" t="inlineStr">
         <is>
           <t>11k維持</t>
         </is>
@@ -1941,12 +1998,15 @@
       <c r="M18" s="8" t="n">
         <v>0.37</v>
       </c>
-      <c r="N18" s="4" t="inlineStr">
+      <c r="N18" s="5" t="n">
+        <v>13000</v>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
         <is>
           <t>✅黒字維持（7/27判定）</t>
         </is>
       </c>
-      <c r="O18" s="4" t="inlineStr">
+      <c r="P18" s="4" t="inlineStr">
         <is>
           <t>13k維持</t>
         </is>
@@ -1988,12 +2048,13 @@
       <c r="K19" s="9" t="inlineStr"/>
       <c r="L19" s="9" t="inlineStr"/>
       <c r="M19" s="9" t="inlineStr"/>
-      <c r="N19" s="9" t="inlineStr">
+      <c r="N19" s="9" t="inlineStr"/>
+      <c r="O19" s="9" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="O19" s="9" t="inlineStr">
+      <c r="P19" s="9" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -2033,12 +2094,13 @@
       <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" s="4" t="inlineStr">
+      <c r="N20" s="4" t="inlineStr"/>
+      <c r="O20" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="O20" s="4" t="inlineStr">
+      <c r="P20" s="4" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -2078,12 +2140,13 @@
       <c r="K21" s="9" t="inlineStr"/>
       <c r="L21" s="9" t="inlineStr"/>
       <c r="M21" s="9" t="inlineStr"/>
-      <c r="N21" s="9" t="inlineStr">
+      <c r="N21" s="9" t="inlineStr"/>
+      <c r="O21" s="9" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="O21" s="9" t="inlineStr">
+      <c r="P21" s="9" t="inlineStr">
         <is>
           <t>−</t>
         </is>
@@ -2131,12 +2194,15 @@
       <c r="M22" s="8" t="n">
         <v>0.03</v>
       </c>
-      <c r="N22" s="4" t="inlineStr">
+      <c r="N22" s="5" t="n">
+        <v>6500</v>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
         <is>
           <t>🔧段階②判定は7/26</t>
         </is>
       </c>
-      <c r="O22" s="4" t="inlineStr">
+      <c r="P22" s="4" t="inlineStr">
         <is>
           <t>6.5k維持</t>
         </is>
@@ -2182,12 +2248,15 @@
       <c r="M23" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="N23" s="9" t="inlineStr">
+      <c r="N23" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="O23" s="9" t="inlineStr">
         <is>
           <t>🔧CRシェア58%獲得（7/29判定）</t>
         </is>
       </c>
-      <c r="O23" s="9" t="inlineStr">
+      <c r="P23" s="9" t="inlineStr">
         <is>
           <t>5k維持</t>
         </is>
@@ -2235,12 +2304,15 @@
       <c r="M24" s="8" t="n">
         <v>-0.08</v>
       </c>
-      <c r="N24" s="4" t="inlineStr">
+      <c r="N24" s="5" t="n">
+        <v>12000</v>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
         <is>
           <t>🔧全開放テスト中（8/6判定）</t>
         </is>
       </c>
-      <c r="O24" s="4" t="inlineStr">
+      <c r="P24" s="4" t="inlineStr">
         <is>
           <t>6k+6k維持</t>
         </is>
@@ -2288,12 +2360,15 @@
       <c r="M25" s="12" t="n">
         <v>-0.22</v>
       </c>
-      <c r="N25" s="9" t="inlineStr">
+      <c r="N25" s="10" t="n">
+        <v>10000</v>
+      </c>
+      <c r="O25" s="9" t="inlineStr">
         <is>
           <t>🔧複製リセット中（7/30判定）</t>
         </is>
       </c>
-      <c r="O25" s="9" t="inlineStr">
+      <c r="P25" s="9" t="inlineStr">
         <is>
           <t>10k維持</t>
         </is>
@@ -2333,12 +2408,13 @@
       <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="4" t="inlineStr"/>
       <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" s="4" t="inlineStr">
+      <c r="N26" s="4" t="inlineStr"/>
+      <c r="O26" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="O26" s="4" t="inlineStr">
+      <c r="P26" s="4" t="inlineStr">
         <is>
           <t>−</t>
         </is>

</xml_diff>

<commit_message>
Excel: yellow-highlight prior-day margin below 30 percent
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-07-24.xlsx
+++ b/data/reports/report-2026-07-24.xlsx
@@ -59,7 +59,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +74,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F6FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2A8"/>
       </patternFill>
     </fill>
   </fills>
@@ -103,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,6 +124,7 @@
     <xf numFmtId="3" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -1436,7 +1442,7 @@
       <c r="G8" s="5" t="n">
         <v>16221</v>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="H8" s="13" t="n">
         <v>0.215</v>
       </c>
       <c r="I8" s="5" t="n">
@@ -1548,7 +1554,7 @@
       <c r="G10" s="5" t="n">
         <v>9742</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="H10" s="13" t="n">
         <v>0.233</v>
       </c>
       <c r="I10" s="5" t="n">
@@ -1660,7 +1666,7 @@
       <c r="G12" s="5" t="n">
         <v>5611</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H12" s="13" t="n">
         <v>0.157</v>
       </c>
       <c r="I12" s="5" t="n">
@@ -1921,10 +1927,10 @@
       <c r="F17" s="10" t="n">
         <v>14940</v>
       </c>
-      <c r="G17" s="13" t="n">
+      <c r="G17" s="14" t="n">
         <v>-923</v>
       </c>
-      <c r="H17" s="11" t="n">
+      <c r="H17" s="13" t="n">
         <v>-0.062</v>
       </c>
       <c r="I17" s="10" t="n">
@@ -1977,10 +1983,10 @@
       <c r="F18" s="5" t="n">
         <v>17940</v>
       </c>
-      <c r="G18" s="14" t="n">
+      <c r="G18" s="15" t="n">
         <v>-1574</v>
       </c>
-      <c r="H18" s="6" t="n">
+      <c r="H18" s="13" t="n">
         <v>-0.08799999999999999</v>
       </c>
       <c r="I18" s="5" t="n">
@@ -2173,10 +2179,10 @@
       <c r="F22" s="5" t="n">
         <v>5980</v>
       </c>
-      <c r="G22" s="14" t="n">
+      <c r="G22" s="15" t="n">
         <v>-2230</v>
       </c>
-      <c r="H22" s="6" t="n">
+      <c r="H22" s="13" t="n">
         <v>-0.373</v>
       </c>
       <c r="I22" s="5" t="n">
@@ -2229,7 +2235,7 @@
       <c r="F23" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="G23" s="13" t="n">
+      <c r="G23" s="14" t="n">
         <v>-5232</v>
       </c>
       <c r="H23" s="9" t="inlineStr"/>
@@ -2277,19 +2283,19 @@
       <c r="D24" s="5" t="n">
         <v>100359</v>
       </c>
-      <c r="E24" s="14" t="n">
+      <c r="E24" s="15" t="n">
         <v>-5658</v>
       </c>
       <c r="F24" s="5" t="n">
         <v>18940</v>
       </c>
-      <c r="G24" s="14" t="n">
+      <c r="G24" s="15" t="n">
         <v>-295</v>
       </c>
-      <c r="H24" s="6" t="n">
+      <c r="H24" s="13" t="n">
         <v>-0.016</v>
       </c>
-      <c r="I24" s="14" t="n">
+      <c r="I24" s="15" t="n">
         <v>-14886</v>
       </c>
       <c r="J24" s="5" t="n">
@@ -2333,19 +2339,19 @@
       <c r="D25" s="10" t="n">
         <v>89191</v>
       </c>
-      <c r="E25" s="13" t="n">
+      <c r="E25" s="14" t="n">
         <v>-12191</v>
       </c>
       <c r="F25" s="10" t="n">
         <v>8980</v>
       </c>
-      <c r="G25" s="13" t="n">
+      <c r="G25" s="14" t="n">
         <v>-6176</v>
       </c>
-      <c r="H25" s="11" t="n">
+      <c r="H25" s="13" t="n">
         <v>-0.6879999999999999</v>
       </c>
-      <c r="I25" s="13" t="n">
+      <c r="I25" s="14" t="n">
         <v>-18790</v>
       </c>
       <c r="J25" s="10" t="n">

</xml_diff>